<commit_message>
Clean up after Github corrections
</commit_message>
<xml_diff>
--- a/data/leaf_temperatures.xlsx
+++ b/data/leaf_temperatures.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10910"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Joe/Documents/College/02- R code/heating/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Joe/Documents/College/02- R code/heating/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5452990-E01B-744F-BA8C-88E7DC879261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{10DC7345-AA72-C246-988E-30A98E654015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-35940" yWindow="760" windowWidth="28800" windowHeight="15800" xr2:uid="{0D1DAA0C-3E7A-A94D-99AC-B432AD39DBD7}"/>
   </bookViews>
@@ -12498,6 +12498,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008F3A2D606D2A7F41B72D5682D1CD7008" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d76c20a2b3afad6e4ced79b91df906ab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="48b2884d-86bd-41bc-b5ea-f3a63e495149" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7e8f2e6da924d638fc8dc52abe2ab2bf" ns2:_="">
     <xsd:import namespace="48b2884d-86bd-41bc-b5ea-f3a63e495149"/>
@@ -12629,22 +12644,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9CB64D7-F540-4BAF-99C7-751D0C161C11}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06BFB0FA-CD1A-4F5C-B895-89C67E76B7DE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7DAC2BA-C817-4ECF-8DFA-94F5C2AE87D4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12660,21 +12677,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9CB64D7-F540-4BAF-99C7-751D0C161C11}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06BFB0FA-CD1A-4F5C-B895-89C67E76B7DE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Commits after in person work
</commit_message>
<xml_diff>
--- a/data/leaf_temperatures.xlsx
+++ b/data/leaf_temperatures.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Joe/Documents/College/02- R code/2- heating/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7F5A7E-B768-2D4D-BBBF-DDCCC4FA5B1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01AB5337-6A00-AC44-980D-557A21B7533D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38100" yWindow="260" windowWidth="36160" windowHeight="20460" xr2:uid="{0D1DAA0C-3E7A-A94D-99AC-B432AD39DBD7}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15740" activeTab="1" xr2:uid="{0D1DAA0C-3E7A-A94D-99AC-B432AD39DBD7}"/>
   </bookViews>
   <sheets>
     <sheet name="temperatures" sheetId="5" r:id="rId1"/>
-    <sheet name="Read Me" sheetId="6" r:id="rId2"/>
+    <sheet name="highest_temps" sheetId="7" r:id="rId2"/>
+    <sheet name="Read Me" sheetId="6" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">temperatures!$A$1:$H$497</definedName>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="28">
   <si>
     <t>Liriodendron tulipifera</t>
   </si>
@@ -12429,6 +12430,151 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58DB13DA-F838-5846-BECE-6E196FC6D268}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1">
+        <v>2022</v>
+      </c>
+      <c r="C1">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>38.799999999999997</v>
+      </c>
+      <c r="C2" s="2">
+        <v>43.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2">
+        <v>38.9</v>
+      </c>
+      <c r="C3" s="2">
+        <v>38.700000000000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="2">
+        <v>45.3</v>
+      </c>
+      <c r="C4" s="2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2">
+        <v>37.6</v>
+      </c>
+      <c r="C5" s="2">
+        <v>40.799999999999997</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="2">
+        <v>36.5</v>
+      </c>
+      <c r="C6" s="2">
+        <v>38.700000000000003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="2">
+        <v>44.5</v>
+      </c>
+      <c r="C7" s="2">
+        <v>44.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="2">
+        <v>40.6</v>
+      </c>
+      <c r="C8" s="2">
+        <v>40.700000000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="2">
+        <v>40.200000000000003</v>
+      </c>
+      <c r="C9" s="2">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="2">
+        <v>45.7</v>
+      </c>
+      <c r="C10" s="2">
+        <v>43.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="2">
+        <v>41.9</v>
+      </c>
+      <c r="C11" s="2">
+        <v>45.3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="2">
+        <v>45.9</v>
+      </c>
+      <c r="C12" s="2">
+        <v>42.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFD35868-CDA1-6442-B101-D76AB4DBCDD5}">
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -12629,18 +12775,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -12662,18 +12808,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9CB64D7-F540-4BAF-99C7-751D0C161C11}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06BFB0FA-CD1A-4F5C-B895-89C67E76B7DE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9CB64D7-F540-4BAF-99C7-751D0C161C11}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updates ahead of meeting
</commit_message>
<xml_diff>
--- a/data/leaf_temperatures.xlsx
+++ b/data/leaf_temperatures.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Joe/Documents/College/02- R code/2- heating/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01AB5337-6A00-AC44-980D-557A21B7533D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BD061F2-4505-1B40-8BA2-91B6595E7285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15740" activeTab="1" xr2:uid="{0D1DAA0C-3E7A-A94D-99AC-B432AD39DBD7}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="29">
   <si>
     <t>Liriodendron tulipifera</t>
   </si>
@@ -61,9 +61,6 @@
   </si>
   <si>
     <t>Celtis laevigata</t>
-  </si>
-  <si>
-    <t>Ulmus americana</t>
   </si>
   <si>
     <t>Juglans nigra</t>
@@ -124,6 +121,12 @@
   </si>
   <si>
     <t>date</t>
+  </si>
+  <si>
+    <t>Ulmus rubra</t>
+  </si>
+  <si>
+    <t>leaf_temp</t>
   </si>
 </sst>
 </file>
@@ -520,28 +523,28 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>21</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>22</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="I1" s="2"/>
     </row>
@@ -1018,7 +1021,7 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B20" s="7">
         <v>44747</v>
@@ -1043,7 +1046,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B21" s="7">
         <v>44747</v>
@@ -1068,7 +1071,7 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B22" s="7">
         <v>44747</v>
@@ -1093,7 +1096,7 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B23" s="7">
         <v>44747</v>
@@ -1118,7 +1121,7 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B24" s="7">
         <v>44747</v>
@@ -1143,7 +1146,7 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B25" s="7">
         <v>44747</v>
@@ -1168,7 +1171,7 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B26" s="7">
         <v>44747</v>
@@ -1193,7 +1196,7 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B27" s="7">
         <v>44747</v>
@@ -1218,7 +1221,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B28" s="7">
         <v>44747</v>
@@ -1243,7 +1246,7 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B29" s="7">
         <v>44747</v>
@@ -1268,7 +1271,7 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B30" s="7">
         <v>44747</v>
@@ -1293,7 +1296,7 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B31" s="7">
         <v>44747</v>
@@ -1318,7 +1321,7 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B32" s="7">
         <v>44747</v>
@@ -1343,7 +1346,7 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B33" s="7">
         <v>44747</v>
@@ -1368,7 +1371,7 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B34" s="7">
         <v>44747</v>
@@ -1393,7 +1396,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B35" s="7">
         <v>44747</v>
@@ -1418,7 +1421,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B36" s="7">
         <v>44747</v>
@@ -1443,7 +1446,7 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B37" s="7">
         <v>44747</v>
@@ -1918,7 +1921,7 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B56" s="7">
         <v>44747</v>
@@ -1943,7 +1946,7 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B57" s="7">
         <v>44747</v>
@@ -1968,7 +1971,7 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B58" s="7">
         <v>44747</v>
@@ -1993,7 +1996,7 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B59" s="7">
         <v>44747</v>
@@ -2018,7 +2021,7 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B60" s="7">
         <v>44747</v>
@@ -2043,7 +2046,7 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B61" s="7">
         <v>44747</v>
@@ -2068,7 +2071,7 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B62" s="7">
         <v>44747</v>
@@ -2093,7 +2096,7 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B63" s="7">
         <v>44747</v>
@@ -2118,7 +2121,7 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B64" s="7">
         <v>44747</v>
@@ -2818,7 +2821,7 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B92" s="7">
         <v>44747</v>
@@ -2843,7 +2846,7 @@
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B93" s="7">
         <v>44747</v>
@@ -2868,7 +2871,7 @@
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B94" s="7">
         <v>44747</v>
@@ -2893,7 +2896,7 @@
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B95" s="7">
         <v>44747</v>
@@ -2918,7 +2921,7 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B96" s="7">
         <v>44747</v>
@@ -2943,7 +2946,7 @@
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B97" s="7">
         <v>44747</v>
@@ -2968,7 +2971,7 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B98" s="7">
         <v>44747</v>
@@ -2993,7 +2996,7 @@
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B99" s="7">
         <v>44747</v>
@@ -3018,7 +3021,7 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B100" s="7">
         <v>44747</v>
@@ -3493,7 +3496,7 @@
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B119" s="7">
         <v>44754</v>
@@ -3518,7 +3521,7 @@
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B120" s="7">
         <v>44754</v>
@@ -3543,7 +3546,7 @@
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B121" s="7">
         <v>44754</v>
@@ -3568,7 +3571,7 @@
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B122" s="7">
         <v>44754</v>
@@ -3593,7 +3596,7 @@
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B123" s="7">
         <v>44754</v>
@@ -3618,7 +3621,7 @@
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B124" s="7">
         <v>44754</v>
@@ -3643,7 +3646,7 @@
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B125" s="7">
         <v>44754</v>
@@ -3668,7 +3671,7 @@
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B126" s="7">
         <v>44754</v>
@@ -3693,7 +3696,7 @@
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B127" s="7">
         <v>44754</v>
@@ -3718,7 +3721,7 @@
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B128" s="7">
         <v>44754</v>
@@ -3743,7 +3746,7 @@
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B129" s="7">
         <v>44754</v>
@@ -3768,7 +3771,7 @@
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B130" s="7">
         <v>44754</v>
@@ -3793,7 +3796,7 @@
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B131" s="7">
         <v>44754</v>
@@ -3818,7 +3821,7 @@
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B132" s="7">
         <v>44754</v>
@@ -3843,7 +3846,7 @@
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B133" s="7">
         <v>44754</v>
@@ -3868,7 +3871,7 @@
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B134" s="7">
         <v>44754</v>
@@ -3893,7 +3896,7 @@
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B135" s="7">
         <v>44754</v>
@@ -3918,7 +3921,7 @@
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B136" s="7">
         <v>44754</v>
@@ -4393,7 +4396,7 @@
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B155" s="7">
         <v>44754</v>
@@ -4418,7 +4421,7 @@
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B156" s="7">
         <v>44754</v>
@@ -4443,7 +4446,7 @@
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B157" s="7">
         <v>44754</v>
@@ -4468,7 +4471,7 @@
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B158" s="7">
         <v>44754</v>
@@ -4493,7 +4496,7 @@
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B159" s="7">
         <v>44754</v>
@@ -4518,7 +4521,7 @@
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B160" s="7">
         <v>44754</v>
@@ -4543,7 +4546,7 @@
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B161" s="7">
         <v>44754</v>
@@ -4568,7 +4571,7 @@
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B162" s="7">
         <v>44754</v>
@@ -4593,7 +4596,7 @@
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B163" s="7">
         <v>44754</v>
@@ -5293,7 +5296,7 @@
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A191" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B191" s="7">
         <v>44754</v>
@@ -5318,7 +5321,7 @@
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A192" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B192" s="7">
         <v>44754</v>
@@ -5343,7 +5346,7 @@
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A193" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B193" s="7">
         <v>44754</v>
@@ -5368,7 +5371,7 @@
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A194" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B194" s="7">
         <v>44754</v>
@@ -5393,7 +5396,7 @@
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A195" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B195" s="7">
         <v>44754</v>
@@ -5418,7 +5421,7 @@
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A196" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B196" s="7">
         <v>44754</v>
@@ -5443,7 +5446,7 @@
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A197" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B197" s="7">
         <v>44754</v>
@@ -5468,7 +5471,7 @@
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A198" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B198" s="7">
         <v>44754</v>
@@ -5493,7 +5496,7 @@
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A199" s="1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B199" s="7">
         <v>44754</v>
@@ -5968,7 +5971,7 @@
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A218" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B218" s="7">
         <v>44756</v>
@@ -5993,7 +5996,7 @@
     </row>
     <row r="219" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A219" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B219" s="7">
         <v>44756</v>
@@ -6018,7 +6021,7 @@
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A220" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B220" s="7">
         <v>44756</v>
@@ -6043,7 +6046,7 @@
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A221" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B221" s="7">
         <v>44756</v>
@@ -6068,7 +6071,7 @@
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A222" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B222" s="7">
         <v>44756</v>
@@ -6093,7 +6096,7 @@
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A223" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B223" s="7">
         <v>44756</v>
@@ -6118,7 +6121,7 @@
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A224" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B224" s="7">
         <v>44756</v>
@@ -6143,7 +6146,7 @@
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A225" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B225" s="7">
         <v>44756</v>
@@ -6168,7 +6171,7 @@
     </row>
     <row r="226" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A226" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B226" s="7">
         <v>44756</v>
@@ -6193,7 +6196,7 @@
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A227" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B227" s="7">
         <v>44756</v>
@@ -6217,7 +6220,7 @@
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A228" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B228" s="7">
         <v>44756</v>
@@ -6241,7 +6244,7 @@
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A229" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B229" s="7">
         <v>44756</v>
@@ -6266,7 +6269,7 @@
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A230" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B230" s="7">
         <v>44756</v>
@@ -6291,7 +6294,7 @@
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A231" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B231" s="7">
         <v>44756</v>
@@ -6316,7 +6319,7 @@
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A232" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B232" s="7">
         <v>44756</v>
@@ -6341,7 +6344,7 @@
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A233" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B233" s="7">
         <v>44756</v>
@@ -6366,7 +6369,7 @@
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A234" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B234" s="7">
         <v>44756</v>
@@ -6390,7 +6393,7 @@
     </row>
     <row r="235" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A235" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B235" s="7">
         <v>44756</v>
@@ -6828,7 +6831,7 @@
     </row>
     <row r="254" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A254" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B254" s="7">
         <v>44756</v>
@@ -6851,7 +6854,7 @@
     </row>
     <row r="255" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A255" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B255" s="7">
         <v>44756</v>
@@ -6874,7 +6877,7 @@
     </row>
     <row r="256" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A256" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B256" s="7">
         <v>44756</v>
@@ -6897,7 +6900,7 @@
     </row>
     <row r="257" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A257" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B257" s="7">
         <v>44756</v>
@@ -6920,7 +6923,7 @@
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A258" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B258" s="7">
         <v>44756</v>
@@ -6943,7 +6946,7 @@
     </row>
     <row r="259" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A259" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B259" s="7">
         <v>44756</v>
@@ -6966,7 +6969,7 @@
     </row>
     <row r="260" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A260" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B260" s="7">
         <v>44756</v>
@@ -6989,7 +6992,7 @@
     </row>
     <row r="261" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A261" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B261" s="7">
         <v>44756</v>
@@ -7012,7 +7015,7 @@
     </row>
     <row r="262" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A262" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B262" s="7">
         <v>44756</v>
@@ -7656,7 +7659,7 @@
     </row>
     <row r="290" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A290" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B290" s="7">
         <v>44756</v>
@@ -7679,7 +7682,7 @@
     </row>
     <row r="291" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A291" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B291" s="7">
         <v>44756</v>
@@ -7702,7 +7705,7 @@
     </row>
     <row r="292" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A292" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B292" s="7">
         <v>44756</v>
@@ -7725,7 +7728,7 @@
     </row>
     <row r="293" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A293" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B293" s="7">
         <v>44756</v>
@@ -7748,7 +7751,7 @@
     </row>
     <row r="294" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A294" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B294" s="7">
         <v>44756</v>
@@ -7771,7 +7774,7 @@
     </row>
     <row r="295" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A295" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B295" s="7">
         <v>44756</v>
@@ -7794,7 +7797,7 @@
     </row>
     <row r="296" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A296" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B296" s="7">
         <v>44756</v>
@@ -7817,7 +7820,7 @@
     </row>
     <row r="297" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A297" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B297" s="7">
         <v>44756</v>
@@ -7840,7 +7843,7 @@
     </row>
     <row r="298" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A298" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B298" s="7">
         <v>44756</v>
@@ -8277,7 +8280,7 @@
     </row>
     <row r="317" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A317" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B317" s="7">
         <v>45161</v>
@@ -8295,12 +8298,12 @@
         <v>4</v>
       </c>
       <c r="H317" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="318" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A318" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B318" s="7">
         <v>45161</v>
@@ -8318,12 +8321,12 @@
         <v>4</v>
       </c>
       <c r="H318" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="319" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A319" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B319" s="7">
         <v>45161</v>
@@ -8341,12 +8344,12 @@
         <v>4</v>
       </c>
       <c r="H319" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="320" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A320" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B320" s="7">
         <v>45161</v>
@@ -8364,12 +8367,12 @@
         <v>4</v>
       </c>
       <c r="H320" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="321" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A321" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B321" s="7">
         <v>45161</v>
@@ -8387,12 +8390,12 @@
         <v>4</v>
       </c>
       <c r="H321" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="322" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A322" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B322" s="7">
         <v>45161</v>
@@ -8410,12 +8413,12 @@
         <v>4</v>
       </c>
       <c r="H322" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="323" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A323" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B323" s="7">
         <v>45161</v>
@@ -8433,12 +8436,12 @@
         <v>4</v>
       </c>
       <c r="H323" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="324" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A324" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B324" s="7">
         <v>45161</v>
@@ -8456,12 +8459,12 @@
         <v>4</v>
       </c>
       <c r="H324" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="325" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A325" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B325" s="7">
         <v>45161</v>
@@ -8479,12 +8482,12 @@
         <v>4</v>
       </c>
       <c r="H325" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="326" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A326" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B326" s="7">
         <v>45161</v>
@@ -8507,7 +8510,7 @@
     </row>
     <row r="327" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A327" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B327" s="7">
         <v>45161</v>
@@ -8530,7 +8533,7 @@
     </row>
     <row r="328" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A328" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B328" s="7">
         <v>45161</v>
@@ -8553,7 +8556,7 @@
     </row>
     <row r="329" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A329" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B329" s="7">
         <v>45161</v>
@@ -8576,7 +8579,7 @@
     </row>
     <row r="330" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A330" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B330" s="7">
         <v>45161</v>
@@ -8599,7 +8602,7 @@
     </row>
     <row r="331" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A331" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B331" s="7">
         <v>45161</v>
@@ -8622,7 +8625,7 @@
     </row>
     <row r="332" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A332" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B332" s="7">
         <v>45161</v>
@@ -8645,7 +8648,7 @@
     </row>
     <row r="333" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A333" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B333" s="7">
         <v>45161</v>
@@ -8668,7 +8671,7 @@
     </row>
     <row r="334" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A334" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B334" s="7">
         <v>45161</v>
@@ -9105,7 +9108,7 @@
     </row>
     <row r="353" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A353" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B353" s="7">
         <v>45161</v>
@@ -9128,7 +9131,7 @@
     </row>
     <row r="354" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A354" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B354" s="7">
         <v>45161</v>
@@ -9151,7 +9154,7 @@
     </row>
     <row r="355" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A355" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B355" s="7">
         <v>45161</v>
@@ -9174,7 +9177,7 @@
     </row>
     <row r="356" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A356" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B356" s="7">
         <v>45161</v>
@@ -9197,7 +9200,7 @@
     </row>
     <row r="357" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A357" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B357" s="7">
         <v>45161</v>
@@ -9220,7 +9223,7 @@
     </row>
     <row r="358" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A358" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B358" s="7">
         <v>45161</v>
@@ -9243,7 +9246,7 @@
     </row>
     <row r="359" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A359" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B359" s="7">
         <v>45161</v>
@@ -9266,7 +9269,7 @@
     </row>
     <row r="360" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A360" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B360" s="7">
         <v>45161</v>
@@ -9289,7 +9292,7 @@
     </row>
     <row r="361" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A361" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B361" s="7">
         <v>45161</v>
@@ -9933,7 +9936,7 @@
     </row>
     <row r="389" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A389" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B389" s="7">
         <v>45161</v>
@@ -9956,7 +9959,7 @@
     </row>
     <row r="390" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A390" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B390" s="7">
         <v>45161</v>
@@ -9979,7 +9982,7 @@
     </row>
     <row r="391" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A391" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B391" s="7">
         <v>45161</v>
@@ -10002,7 +10005,7 @@
     </row>
     <row r="392" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A392" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B392" s="7">
         <v>45161</v>
@@ -10025,7 +10028,7 @@
     </row>
     <row r="393" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A393" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B393" s="7">
         <v>45161</v>
@@ -10048,7 +10051,7 @@
     </row>
     <row r="394" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A394" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B394" s="7">
         <v>45161</v>
@@ -10071,7 +10074,7 @@
     </row>
     <row r="395" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A395" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B395" s="7">
         <v>45161</v>
@@ -10094,7 +10097,7 @@
     </row>
     <row r="396" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A396" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B396" s="7">
         <v>45161</v>
@@ -10117,7 +10120,7 @@
     </row>
     <row r="397" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A397" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B397" s="7">
         <v>45161</v>
@@ -10554,7 +10557,7 @@
     </row>
     <row r="416" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A416" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B416" s="7">
         <v>45163</v>
@@ -10577,7 +10580,7 @@
     </row>
     <row r="417" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A417" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B417" s="7">
         <v>45163</v>
@@ -10600,7 +10603,7 @@
     </row>
     <row r="418" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A418" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B418" s="7">
         <v>45163</v>
@@ -10623,7 +10626,7 @@
     </row>
     <row r="419" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A419" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B419" s="7">
         <v>45163</v>
@@ -10646,7 +10649,7 @@
     </row>
     <row r="420" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A420" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B420" s="7">
         <v>45163</v>
@@ -10669,7 +10672,7 @@
     </row>
     <row r="421" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A421" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B421" s="7">
         <v>45163</v>
@@ -10692,7 +10695,7 @@
     </row>
     <row r="422" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A422" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B422" s="7">
         <v>45163</v>
@@ -10715,7 +10718,7 @@
     </row>
     <row r="423" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A423" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B423" s="7">
         <v>45163</v>
@@ -10738,7 +10741,7 @@
     </row>
     <row r="424" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A424" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B424" s="7">
         <v>45163</v>
@@ -10761,7 +10764,7 @@
     </row>
     <row r="425" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A425" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B425" s="7">
         <v>45163</v>
@@ -10784,7 +10787,7 @@
     </row>
     <row r="426" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A426" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B426" s="7">
         <v>45163</v>
@@ -10807,7 +10810,7 @@
     </row>
     <row r="427" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A427" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B427" s="7">
         <v>45163</v>
@@ -10830,7 +10833,7 @@
     </row>
     <row r="428" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A428" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B428" s="7">
         <v>45163</v>
@@ -10853,7 +10856,7 @@
     </row>
     <row r="429" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A429" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B429" s="7">
         <v>45163</v>
@@ -10876,7 +10879,7 @@
     </row>
     <row r="430" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A430" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B430" s="7">
         <v>45163</v>
@@ -10899,7 +10902,7 @@
     </row>
     <row r="431" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A431" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B431" s="7">
         <v>45163</v>
@@ -10922,7 +10925,7 @@
     </row>
     <row r="432" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A432" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B432" s="7">
         <v>45163</v>
@@ -10945,7 +10948,7 @@
     </row>
     <row r="433" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A433" s="5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B433" s="7">
         <v>45163</v>
@@ -11382,7 +11385,7 @@
     </row>
     <row r="452" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A452" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B452" s="7">
         <v>45163</v>
@@ -11405,7 +11408,7 @@
     </row>
     <row r="453" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A453" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B453" s="7">
         <v>45163</v>
@@ -11428,7 +11431,7 @@
     </row>
     <row r="454" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A454" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B454" s="7">
         <v>45163</v>
@@ -11451,7 +11454,7 @@
     </row>
     <row r="455" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A455" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B455" s="7">
         <v>45163</v>
@@ -11474,7 +11477,7 @@
     </row>
     <row r="456" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A456" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B456" s="7">
         <v>45163</v>
@@ -11497,7 +11500,7 @@
     </row>
     <row r="457" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A457" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B457" s="7">
         <v>45163</v>
@@ -11520,7 +11523,7 @@
     </row>
     <row r="458" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A458" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B458" s="7">
         <v>45163</v>
@@ -11543,7 +11546,7 @@
     </row>
     <row r="459" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A459" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B459" s="7">
         <v>45163</v>
@@ -11566,7 +11569,7 @@
     </row>
     <row r="460" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A460" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B460" s="7">
         <v>45163</v>
@@ -12210,7 +12213,7 @@
     </row>
     <row r="488" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A488" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B488" s="7">
         <v>45163</v>
@@ -12233,7 +12236,7 @@
     </row>
     <row r="489" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A489" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B489" s="7">
         <v>45163</v>
@@ -12256,7 +12259,7 @@
     </row>
     <row r="490" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A490" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B490" s="7">
         <v>45163</v>
@@ -12279,7 +12282,7 @@
     </row>
     <row r="491" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A491" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B491" s="7">
         <v>45163</v>
@@ -12302,7 +12305,7 @@
     </row>
     <row r="492" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A492" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B492" s="7">
         <v>45163</v>
@@ -12325,7 +12328,7 @@
     </row>
     <row r="493" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A493" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B493" s="7">
         <v>45163</v>
@@ -12348,7 +12351,7 @@
     </row>
     <row r="494" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A494" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B494" s="7">
         <v>45163</v>
@@ -12371,7 +12374,7 @@
     </row>
     <row r="495" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A495" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B495" s="7">
         <v>45163</v>
@@ -12394,7 +12397,7 @@
     </row>
     <row r="496" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A496" s="5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B496" s="7">
         <v>45163</v>
@@ -12431,141 +12434,263 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58DB13DA-F838-5846-BECE-6E196FC6D268}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1">
-        <v>2022</v>
-      </c>
-      <c r="C1">
-        <v>2023</v>
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2">
+        <v>2022</v>
+      </c>
+      <c r="C2" s="2">
         <v>38.799999999999997</v>
-      </c>
-      <c r="C2" s="2">
-        <v>43.5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3">
+        <v>2022</v>
+      </c>
+      <c r="C3" s="2">
         <v>38.9</v>
-      </c>
-      <c r="C3" s="2">
-        <v>38.700000000000003</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="2">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>2022</v>
+      </c>
+      <c r="C4" s="2">
         <v>45.3</v>
-      </c>
-      <c r="C4" s="2">
-        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="2">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>2022</v>
+      </c>
+      <c r="C5" s="2">
         <v>37.6</v>
-      </c>
-      <c r="C5" s="2">
-        <v>40.799999999999997</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
+        <v>2022</v>
+      </c>
+      <c r="C6" s="2">
         <v>36.5</v>
-      </c>
-      <c r="C6" s="2">
-        <v>38.700000000000003</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7">
+        <v>2022</v>
+      </c>
+      <c r="C7" s="2">
         <v>44.5</v>
-      </c>
-      <c r="C7" s="2">
-        <v>44.8</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="2">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>2022</v>
+      </c>
+      <c r="C8" s="2">
         <v>40.6</v>
-      </c>
-      <c r="C8" s="2">
-        <v>40.700000000000003</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9">
+        <v>2022</v>
+      </c>
+      <c r="C9" s="2">
         <v>40.200000000000003</v>
-      </c>
-      <c r="C9" s="2">
-        <v>39.5</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10">
+        <v>2022</v>
+      </c>
+      <c r="C10" s="2">
         <v>45.7</v>
-      </c>
-      <c r="C10" s="2">
-        <v>43.5</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11">
+        <v>2022</v>
+      </c>
+      <c r="C11" s="2">
         <v>41.9</v>
-      </c>
-      <c r="C11" s="2">
-        <v>45.3</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" s="2">
+        <v>27</v>
+      </c>
+      <c r="B12">
+        <v>2022</v>
+      </c>
+      <c r="C12" s="2">
         <v>45.9</v>
       </c>
-      <c r="C12" s="2">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B13">
+        <v>2023</v>
+      </c>
+      <c r="C13" s="2">
+        <v>43.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14">
+        <v>2023</v>
+      </c>
+      <c r="C14" s="2">
+        <v>38.700000000000003</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15">
+        <v>2023</v>
+      </c>
+      <c r="C15" s="2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16">
+        <v>2023</v>
+      </c>
+      <c r="C16" s="2">
+        <v>40.799999999999997</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>2</v>
+      </c>
+      <c r="B17">
+        <v>2023</v>
+      </c>
+      <c r="C17" s="2">
+        <v>38.700000000000003</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18">
+        <v>2023</v>
+      </c>
+      <c r="C18" s="2">
+        <v>44.8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19">
+        <v>2023</v>
+      </c>
+      <c r="C19" s="2">
+        <v>40.700000000000003</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20">
+        <v>2023</v>
+      </c>
+      <c r="C20" s="2">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21">
+        <v>2023</v>
+      </c>
+      <c r="C21" s="2">
+        <v>43.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22">
+        <v>2023</v>
+      </c>
+      <c r="C22" s="2">
+        <v>45.3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23">
+        <v>2023</v>
+      </c>
+      <c r="C23" s="2">
         <v>42.1</v>
       </c>
     </row>
@@ -12584,17 +12709,17 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -12602,7 +12727,7 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -12610,7 +12735,7 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -12618,7 +12743,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -12626,7 +12751,7 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -12634,7 +12759,7 @@
         <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -12643,6 +12768,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008F3A2D606D2A7F41B72D5682D1CD7008" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d76c20a2b3afad6e4ced79b91df906ab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="48b2884d-86bd-41bc-b5ea-f3a63e495149" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7e8f2e6da924d638fc8dc52abe2ab2bf" ns2:_="">
     <xsd:import namespace="48b2884d-86bd-41bc-b5ea-f3a63e495149"/>
@@ -12774,22 +12914,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9CB64D7-F540-4BAF-99C7-751D0C161C11}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06BFB0FA-CD1A-4F5C-B895-89C67E76B7DE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7DAC2BA-C817-4ECF-8DFA-94F5C2AE87D4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12805,21 +12947,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9CB64D7-F540-4BAF-99C7-751D0C161C11}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06BFB0FA-CD1A-4F5C-B895-89C67E76B7DE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Housekeeping + updates after week's work
</commit_message>
<xml_diff>
--- a/data/leaf_temperatures.xlsx
+++ b/data/leaf_temperatures.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Joe/Documents/College/02- R code/2- heating/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BD061F2-4505-1B40-8BA2-91B6595E7285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01248CE0-91B7-F34F-913F-95A24656A7F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15740" activeTab="1" xr2:uid="{0D1DAA0C-3E7A-A94D-99AC-B432AD39DBD7}"/>
+    <workbookView xWindow="-37640" yWindow="1420" windowWidth="28800" windowHeight="15740" activeTab="1" xr2:uid="{0D1DAA0C-3E7A-A94D-99AC-B432AD39DBD7}"/>
   </bookViews>
   <sheets>
     <sheet name="temperatures" sheetId="5" r:id="rId1"/>
@@ -12768,21 +12768,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008F3A2D606D2A7F41B72D5682D1CD7008" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d76c20a2b3afad6e4ced79b91df906ab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="48b2884d-86bd-41bc-b5ea-f3a63e495149" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7e8f2e6da924d638fc8dc52abe2ab2bf" ns2:_="">
     <xsd:import namespace="48b2884d-86bd-41bc-b5ea-f3a63e495149"/>
@@ -12914,24 +12899,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9CB64D7-F540-4BAF-99C7-751D0C161C11}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06BFB0FA-CD1A-4F5C-B895-89C67E76B7DE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7DAC2BA-C817-4ECF-8DFA-94F5C2AE87D4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12947,4 +12930,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06BFB0FA-CD1A-4F5C-B895-89C67E76B7DE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9CB64D7-F540-4BAF-99C7-751D0C161C11}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>